<commit_message>
Updated Gender related data and locator and Bulk upload excel dates
</commit_message>
<xml_diff>
--- a/test/data/Bulk_Upload_Bookings.xlsx
+++ b/test/data/Bulk_Upload_Bookings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ibase1-my.sharepoint.com/personal/keerthi_kodakandla_qualitestgroup_com/Documents/LL/Automation_LL/Premaster_FinalCopy/ll-ui-test-automation/test/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_A168384FC2E2221AB99B176D47CADDEA62BE7D0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EF42953-6247-4AC0-B782-487476C74BBC}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_A168384FC2E2221AB99B176D47CADDEA62BE7D0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0F9700E-E34B-45D4-B004-D385F6E17532}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1393,7 +1393,7 @@
         <v>51</v>
       </c>
       <c r="B2" s="33">
-        <v>45931</v>
+        <v>47027</v>
       </c>
       <c r="C2" s="34">
         <v>0.375</v>
@@ -1450,7 +1450,7 @@
         <v>56</v>
       </c>
       <c r="B3" s="33">
-        <v>45966</v>
+        <v>47062</v>
       </c>
       <c r="C3" s="34">
         <v>0.4375</v>
@@ -1511,7 +1511,7 @@
         <v>62</v>
       </c>
       <c r="B4" s="33">
-        <v>45967</v>
+        <v>47063</v>
       </c>
       <c r="C4" s="34">
         <v>0.46875</v>

</xml_diff>